<commit_message>
Tracker: completed count 67 -> 75
</commit_message>
<xml_diff>
--- a/docs/FlightPro_Manager_Master_Plan_Tracker.xlsx
+++ b/docs/FlightPro_Manager_Master_Plan_Tracker.xlsx
@@ -740,7 +740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E75"/>
+  <dimension ref="A1:E76"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="22" min="1" max="1"/>
@@ -2688,6 +2688,33 @@
       <c r="E75" s="28" t="inlineStr">
         <is>
           <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="28" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="B76" s="28" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C76" s="29" t="inlineStr">
+        <is>
+          <t>ground_school_enrollment writes moved behind gated server routes (item 39, the last of the 2026-08-24 review's direct-write findings)</t>
+        </is>
+      </c>
+      <c r="D76" s="28" t="inlineStr">
+        <is>
+          <t>Six write sites went straight to Supabase on the public anon key with no role check: four on the Ground School Attendance page (attendance status, five exam fields, add student, remove student) and two in syncGroundSchoolFromChecklist(). The page's RoleGate decided what RENDERED, not what the database accepted. Adds app/api/ground-school/enrollment (POST/PATCH/DELETE, GROUND_SCHOOL_WRITE_ROLES) and app/api/ground-school/checklist-sync (POST, REQUIREMENTS_WRITE_ROLES), both on supabaseAdmin. THE PATCH FIELD WHITELIST IS THE POINT: updateExam() passed an arbitrary column name through as {[field]: value}; a route forwarding that verbatim would be an arbitrary-column-write primitive carrying the SERVICE-ROLE key — worse than what it replaced. Five columns accepted; class_id/student_id excluded so no caller can re-point one student's record onto another. DGCA roll-number rule now enforced server-side too. ROLE SETS PRESERVED EXACTLY — GROUND_SCHOOL_WRITE_ROLES is the attendance page's previously-INLINE array, now shared so page and route cannot drift. This moved WHERE the check happens, not WHO passes it. VERIFIED LIVE 2026-09-16 as dummy.operations: enrollment route ADMITS operations (404 on a missing row = cleared the gate, wrote nothing), checklist-sync REJECTS operations (403) — both directions of the role split proven in one session. Also verified as super_admin: whitelist rejects a bad column (400), six validation paths correct, DGCA guard does a real lookup, checklist-sync lifecycle created/unchanged/deleted. NOT VERIFIED: the attendance page's four UI paths — there are zero ground school classes in the data, so nothing to act on. Route contract + typecheck only.</t>
+        </is>
+      </c>
+      <c r="E76" s="28" t="inlineStr">
+        <is>
+          <t>2026-09-16 (8eaeb6b)</t>
         </is>
       </c>
     </row>
@@ -2705,7 +2732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="22" min="1" max="1"/>
@@ -3249,6 +3276,33 @@
       <c r="E21" s="33" t="inlineStr">
         <is>
           <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="30" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B22" s="30" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C22" s="31" t="inlineStr">
+        <is>
+          <t>Ground School Attendance page still READS ground_school_enrollment directly on the anon key</t>
+        </is>
+      </c>
+      <c r="D22" s="30" t="inlineStr">
+        <is>
+          <t>Writes were closed 2026-09-16 (Completed 75); reads were deliberately left alone rather than smuggled into a writes fix. Same shape as the nine remaining unscoped tables — belongs in that effort, not its own row of work.</t>
+        </is>
+      </c>
+      <c r="E22" s="33" t="inlineStr">
+        <is>
+          <t>Normal</t>
         </is>
       </c>
     </row>
@@ -4350,7 +4404,7 @@
     <row r="2">
       <c r="A2" s="22" t="inlineStr">
         <is>
-          <t>Updated 2026-09-11. Previous update 2026-09-10.</t>
+          <t>Updated 2026-09-16. Previous update 2026-09-11.</t>
         </is>
       </c>
     </row>
@@ -4366,7 +4420,7 @@
       </c>
       <c r="B4" s="39" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>75</t>
         </is>
       </c>
       <c r="D4" s="22" t="inlineStr">
@@ -4383,7 +4437,7 @@
       </c>
       <c r="B5" s="39" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="D5" s="22" t="inlineStr">
@@ -4473,7 +4527,7 @@
     <row r="12" ht="31.5" customHeight="1" s="23">
       <c r="A12" s="42" t="inlineStr">
         <is>
-          <t>SHIPPED: SWR migration (8 stages), Safety Management workflow, squawk reporting, Duty Hours, drag-and-drop rescheduling, RMT/IMT numbering, repo cruft removal, Zustand removal, IST date fixes, NOAA visibility fix, SkyLink NOTAM integration + auth + disclaimer, ConfigTable consolidation, DGCA Maintenance Log, exceljs→write-excel-file, /api/students dedupe, DGCA audit-pack export, quick-reschedule stale-state fix, projected-finish progression (phase 1).</t>
+          <t>SHIPPED: SWR migration (8 stages), Safety Management workflow, squawk reporting, Duty Hours, drag-and-drop rescheduling, RMT/IMT numbering, repo cruft removal, Zustand removal, IST date fixes, NOAA visibility fix, SkyLink NOTAM integration + auth + disclaimer, ConfigTable consolidation, DGCA Maintenance Log, exceljs→write-excel-file, /api/students dedupe, DGCA audit-pack export, quick-reschedule stale-state fix, projected-finish progression (phase 1) ground_school_enrollment gated routes (item 39 closed).</t>
         </is>
       </c>
     </row>

</xml_diff>